<commit_message>
Add new build scripts and documentation for Africa CDC, AUC, and AUDA-NEPAD initiatives. Introduce synchronized output generation for Word, PDF, and PowerPoint formats, ensuring compliance with eligibility criteria and project objectives. Include source of truth files to maintain alignment across deliverables and enhance clarity for applicants.
</commit_message>
<xml_diff>
--- a/opportunities/opportunities.xlsx
+++ b/opportunities/opportunities.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scan Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,10 @@
     <col width="74" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -530,6 +534,26 @@
           <t>Gender Category</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Application Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Submission Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Application Folder</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="92" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -557,6 +581,22 @@
           <t>Gender-based (women/girls)</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>applications/awief</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="92" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -584,6 +624,22 @@
           <t>Gender-based (women/girls)</t>
         </is>
       </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>applications/auc</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="92" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -611,6 +667,22 @@
           <t>Gender-based (women/girls)</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>applications/feminist-ai</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="92" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -638,6 +710,22 @@
           <t>Gender-based (women/girls)</t>
         </is>
       </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>applications/girlcode</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="92" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -665,6 +753,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>applications/auda-srh</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -692,6 +796,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>applications/gadfly</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -719,6 +839,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>applications/dos-uganda</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -746,6 +882,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>applications/whs</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="92" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -773,6 +925,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>applications/oyw</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="92" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -800,6 +968,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>applications/africa-cdc</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="92" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -827,6 +1011,22 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>applications/ifad</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="92" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -854,9 +1054,25 @@
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>applications/govtech</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:I13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -867,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -906,7 +1122,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17 05:32</t>
+          <t>2026-07-17 09:54</t>
         </is>
       </c>
     </row>
@@ -1021,10 +1237,22 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t>Application packs</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Win-win packs (rules + Word/PDF/PPT) live under applications/{slug}/ for every Opportunities row. Status set to Drafting until submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Deadlines and eligibility are quoted from Opportunities for Youth article text. ALWAYS confirm on the official programme page before applying — details can change.</t>
         </is>

</xml_diff>

<commit_message>
Refine FCHIP documentation and enhance application pack generation
- Updated `fairBanks_refined_project_idea.mdc` to clarify the funding ask and emphasize the validation and scaling of the working FCHIP MVP.
- Revised `build_africa-health-tech-accelerator_docs.py` to create a dedicated pitch-deck folder, ensuring organized access to the pitch materials for the application process.
- Improved the application pack documents to reflect the confirmed MVP status and updated submission readiness criteria, reinforcing FairBanks' commitment to effective communication and operational readiness.
</commit_message>
<xml_diff>
--- a/opportunities/opportunities.xlsx
+++ b/opportunities/opportunities.xlsx
@@ -633,7 +633,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>applications/auda-srh</t>
@@ -676,7 +676,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n"/>
+      <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>applications/awief</t>
@@ -696,7 +696,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Six-month pan-African accelerator for early-stage health-tech startups and SMEs. Tracks include digital healthcare, health data and intelligent technologies, prevention/access services, and related innovation. Benefits: structured training, mentorship, seed-funding opportunities, investor Demo Day, and continental visibility. Needs at least two founders, an MVP, and a scale-across-Africa commitment. Excellent near-term fit for FCHIP as a community health intelligence / digital health venture. Deadline extended to 20 July 2026 — apply immediately.</t>
+          <t>Six-month pan-African accelerator for early-stage health-tech startups and SMEs. Tracks include digital healthcare, health data and intelligent technologies, prevention/access services, and related innovation. Benefits: structured training, mentorship, seed-funding opportunities, investor Demo Day, and continental visibility. Needs at least two founders, an MVP, and a scale-across-Africa commitment. Excellent near-term fit for FCHIP (working MVP) as a community health intelligence / digital health venture. Deadline extended to 20 July 2026 — apply immediately.</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -719,8 +719,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="92" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Drafting</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -758,8 +758,12 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>applications/nexa-climate-health</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="92" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -797,7 +801,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>applications/gadfly</t>
@@ -840,7 +844,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n"/>
+      <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
           <t>applications/auc</t>
@@ -883,8 +887,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -922,7 +926,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n"/>
+      <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t>applications/feminist-ai</t>
@@ -965,7 +969,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>applications/dos-uganda</t>
@@ -1008,7 +1012,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n"/>
+      <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t>applications/whs</t>
@@ -1051,7 +1055,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>applications/oyw</t>
@@ -1094,8 +1098,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="92" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1133,7 +1137,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>applications/africa-cdc</t>
@@ -1176,8 +1180,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="10" t="n"/>
+      <c r="H15" s="10" t="inlineStr"/>
+      <c r="I15" s="10" t="inlineStr"/>
     </row>
     <row r="16" ht="92" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -1215,8 +1219,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
@@ -1254,8 +1258,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H17" s="12" t="n"/>
-      <c r="I17" s="12" t="n"/>
+      <c r="H17" s="12" t="inlineStr"/>
+      <c r="I17" s="12" t="inlineStr"/>
     </row>
     <row r="18" ht="92" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -1293,8 +1297,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="92" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1332,7 +1336,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H19" s="4" t="n"/>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
           <t>applications/ifad</t>
@@ -1375,7 +1379,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n"/>
+      <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>applications/girlcode</t>
@@ -1418,86 +1422,86 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n"/>
+      <c r="H21" s="10" t="inlineStr"/>
+      <c r="I21" s="10" t="inlineStr"/>
     </row>
     <row r="22" ht="92" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>DIV Fund (Development Innovation Ventures) — Open Innovation Grants</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.div.fund/apply</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Evidence-driven open innovation fund accepting applications year-round. Stages roughly: Pilot up to ~US$200,000; Testing higher; Scale up to about US$1.5 million. Funds innovations that can cost-effectively improve millions of lives in low- and middle-income countries. Open to nonprofits, startups, universities, and social enterprises — Ugandan applicants eligible. Good medium-term pathway for FCHIP if you can show a clear pilot plan, cost-effectiveness case, and path to scale across peri-urban and district health systems.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Rolling (applications accepted year-round)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="92" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>AFNet Flexible Grant (African Women for Change Network)</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>https://afwcnet.org/women-grants</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Small flexible grant (about US$5,000) for women leaders and women-led organisations driving community change in Africa. Reviewed on a rolling basis. Useful seed support for a woman-led FairBanks Community Reach or FCHIP pilot activity in peri-urban Kampala communities (outreach, maternal support, or CHW coordination). Confirm current application steps and eligibility on the AFNet channel before applying; listing details can change.</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Rolling</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Gender-based (women/girls)</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="n"/>
-      <c r="I22" s="8" t="n"/>
-    </row>
-    <row r="23" ht="92" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>DIV Fund (Development Innovation Ventures) — Open Innovation Grants</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>https://www.div.fund/apply</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Evidence-driven open innovation fund accepting applications year-round. Stages roughly: Pilot up to ~US$200,000; Testing higher; Scale up to about US$1.5 million. Funds innovations that can cost-effectively improve millions of lives in low- and middle-income countries. Open to nonprofits, startups, universities, and social enterprises — Ugandan applicants eligible. Good medium-term pathway for FCHIP if you can show a clear pilot plan, cost-effectiveness case, and path to scale across peri-urban and district health systems.</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Rolling (applications accepted year-round)</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Multi-gender (all genders)</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
     </row>
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -1535,8 +1539,8 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="92" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1574,7 +1578,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H25" s="4" t="n"/>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
           <t>applications/govtech</t>
@@ -1593,11 +1597,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="118" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1612,19 +1616,19 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Merged on</t>
+          <t>Scanned on</t>
         </is>
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>2026-07-19 21:46</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
+          <t>2026-07-20 13:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Document type</t>
@@ -1632,11 +1636,11 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Merged tracker: opportunities.xlsx + former opportunities_periurban_fchip_2026-07.xlsx. Deduped by title/URL. Sorted by earliest Application Deadline (rolling/unknown last). Peri-urban row highlight colours preserved (green / blue / red / black).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+          <t>Canonical merged tracker (OFY scan + former peri-urban / FCHIP complementary scan). Sorted by earliest Application Deadline; rolling/unknown last. Peri-urban highlight colours preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Applicant context</t>
@@ -1644,11 +1648,11 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>FairBanks / FCHIP — a Ugandan community health intelligence venture. We are Ugandans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+          <t>FairBanks / FCHIP — a Ugandan community health intelligence venture (peri-urban Kampala communities; CHW/VHT cascade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Sources</t>
@@ -1656,11 +1660,11 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Primary OFY tracker plus peri-urban / FCHIP / community-health deep scan sources (Grand Challenges, IDRC ANeSA, Africa Health ExCon, UN Women SIARP, DIV, FID, EDCTP3, Wellcome Snakebite, Social Shifters, AFNet, Gilead, DRK, and related).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+          <t>Opportunities for Youth plus peri-urban / FCHIP sources (Grand Challenges Nexa, IDRC ANeSA, Africa Health ExCon, UN Women SIARP, DIV, FID, EDCTP3, Wellcome Snakebite, Social Shifters, AFNet, Gilead, DRK, and related).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Eligibility filter</t>
@@ -1668,35 +1672,35 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Still-open (or reopening) calls open to Ugandan applicants (global, pan-African, East Africa, or Uganda-specific).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+          <t>Included ONLY opportunities that are (a) still open (or reopening) and (b) open to Ugandan applicants (global, pan-African / African Union, or Uganda-specific).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
+          <t>Highlight legend</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Green = peri-urban priority women/gender calls. Blue = strong FCHIP / digital / innovation fits. Red = research awards with narrower fit. Black = FID portal reopen watch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
           <t>Gender categories</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Gender-based (women/girls): 6. Multi-gender (all genders): 18. Total: 24.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Highlight legend</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Green = peri-urban priority women/gender calls. Blue = strong FCHIP / digital / innovation fits. Red = research awards with narrower fit. Black = FID portal reopen watch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Priority soon</t>
@@ -1704,11 +1708,11 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>1) Africa Health-Tech Accelerator (20 Jul) 2) Nexa climate–health early warning (22 Jul) 3) UN Women SIARP 2.0 if regional consortium ready (27 Jul) 4) IDRC ANeSA LoI (23 Aug) 5) EDCTP3 digital/AI consortium path (2 Sep) 6) FID portal reopen 1 Sep 7) DIV rolling evidence pathway.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+          <t>Africa Health-Tech Accelerator (20 Jul), Nexa (22 Jul), AWIEF (20 Jul), Gadfly (24 Jul), SIARP 2.0 (27 Jul), US State Dept Uganda SOI / WHS (31 Jul).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Best fit for FairBanks</t>
@@ -1716,67 +1720,31 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>US State Dept Uganda Health MOU, AWIEF Pitch n Grow, WHS Youth Group, Africa CDC AES Fellowship, Gadfly Web App Grant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+          <t>US State Dept Uganda Health MOU, Nexa, Africa Health-Tech Accelerator, AWIEF Pitch n Grow, EDCTP3 DIGIT-02 (consortium), DIV/FID evidence-to-scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Best peri-urban / FCHIP fits</t>
+          <t>Application packs</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Nexa (mosquito-borne early warning for dense peri-urban settlements); Africa Health-Tech Accelerator (FCHIP digital health MVP); EDCTP3 DIGIT-02 (scale/interop of existing CHW/digital tools via consortium); ANeSA (peri-urban adolescent/maternal SRHR research with university partner); DIV/FID (evidence-to-scale); SIARP 2.0 (women/girls SRHR + community accountability if consortium-ready).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
+          <t>Win-win packs (rules + Word/PDF/PPT) live under applications/{slug}/ where an app_slug is set. Status Drafting until submitted; peri-urban adds start as Not started.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Excluded (closed / paused)</t>
+          <t>Important</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>Mak-AI/Zindi Multilingual Health QA (closed ~21 Jun / under code review); SheConnects CARE (8 Jul); Inclusive AI HAIDI (17 Jul); SAFEStart+ Uganda (30 Jun); AmplifyChange Strengthening (16 Jun); Luena Eneko (31 May); la Caixa Child Survival (26 May); UNICEF Climate Ventures (17 May); AUDA-NEPAD HGS / Villgro HGS (19 May); GSMA Green Transition (6 Apr); EVAH Spring RFP (1 Apr); Gates Cost-Disruptive Diagnostics (28 Apr); reach52 Growth Partner Q1 (31 Mar); ACT Foundation (30 Jan); Echoing Green 2026 (closed); AJA Foundation paused; GIF not accepting applications (official site); CDC Uganda health-security NOFO (~25 Jun estimated / closed); UNICEF Uganda Health &amp; HIV CFEI (closed on DevelopmentAid).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Excluded (scam / ineligible)</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>ifcgrants.org Healthcare Access Initiative — FAKE IFC grant site (World Bank/IFC scam warning); Reckitt Catalyst 2026/27 — Uganda not in eligible markets; Mastercard Pathways to Scale — Ethiopia/Ghana/Nigeria/Rwanda only; Africa Health Collaborative Research Fund — no Uganda member university; Gates Pan-Orthoebolavirus Diagnostics — needs BSL-4/high-consequence pathogen diagnostics expertise; Beginnings Fund &amp; Mulago — no unsolicited proposals (monitor partnership/referral paths); Darwin biodiversity; Nigeria/Ethiopia-only CSO funds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Important</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Deadlines and eligibility change quickly. ALWAYS confirm on the official programme page before applying. Never use sites that impersonate IFC/World Bank grant portals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Build script</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Rebuild via opportunities/build_opportunities.py (canonical). Peri-urban companion file removed after merge.</t>
+          <t>ALWAYS confirm deadlines and eligibility on the official programme page before applying. Never use sites that impersonate IFC/World Bank grant portals.</t>
         </is>
       </c>
     </row>

</xml_diff>